<commit_message>
adding certification in gallery dropdown done for both
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -581,9 +581,23 @@
         <v>12th</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>jih iuh</v>
+      </c>
+      <c r="C14" t="str">
+        <v>7687857569</v>
+      </c>
+      <c r="D14" t="str">
+        <v>12th</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
creating .env in frontend
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,9 @@
       <c r="D1" t="str">
         <v>Qualification</v>
       </c>
+      <c r="E1" t="str">
+        <v>AlternatePhone</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -595,9 +598,26 @@
         <v>12th</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>sss</v>
+      </c>
+      <c r="C15" t="str">
+        <v>6666666666</v>
+      </c>
+      <c r="D15" t="str">
+        <v>12th</v>
+      </c>
+      <c r="E15" t="str">
+        <v>7777777777</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
removing space in EMAIL_PASS
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -615,9 +615,26 @@
         <v>7777777777</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>ggg</v>
+      </c>
+      <c r="C16" t="str">
+        <v>9999999999</v>
+      </c>
+      <c r="D16" t="str">
+        <v>12th</v>
+      </c>
+      <c r="E16" t="str">
+        <v>8888888888</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adding alternate no. in mail
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -632,9 +632,26 @@
         <v>8888888888</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>ffff</v>
+      </c>
+      <c r="C17" t="str">
+        <v>6666666666</v>
+      </c>
+      <c r="D17" t="str">
+        <v>12th</v>
+      </c>
+      <c r="E17" t="str">
+        <v>7777777777</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changes in alternate no.
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -649,9 +649,43 @@
         <v>7777777777</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>rahim khan</v>
+      </c>
+      <c r="C18" t="str">
+        <v>9999999999</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Diploma</v>
+      </c>
+      <c r="E18" t="str">
+        <v>7777777777</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>sahil khan</v>
+      </c>
+      <c r="C19" t="str">
+        <v>7777777777</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Diploma</v>
+      </c>
+      <c r="E19" t="str">
+        <v>8888888888</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changes in frontend .env
</commit_message>
<xml_diff>
--- a/backend/enquiries.xlsx
+++ b/backend/enquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -683,9 +683,26 @@
         <v>8888888888</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ismat khanam</v>
+      </c>
+      <c r="C20" t="str">
+        <v>7777777777</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Graduate</v>
+      </c>
+      <c r="E20" t="str">
+        <v>8888888888</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>